<commit_message>
Updated experimental results - Rev1
</commit_message>
<xml_diff>
--- a/results/IRECS_ExperimentalResults.xlsx
+++ b/results/IRECS_ExperimentalResults.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ucordoba-my.sharepoint.com/personal/i72raqua_uco_es/Documents/Documentos/Investigacion/Revistas/2023_G3PSLR/zenodo/results/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\auror\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="6" documentId="11_6632A726173F86BFA6A99C7F85B0EA6376CC8244" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E1FB7FD5-C48E-4C50-8D9F-5536F0CE5BAA}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29C6EB98-E2A8-4BB7-80D9-5099022B4658}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-24810" yWindow="1605" windowWidth="21600" windowHeight="11235" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="2" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="RQ1-ClassifStrategy" sheetId="2" r:id="rId1"/>
@@ -18,6 +18,7 @@
     <sheet name="RQ1-GeneticParams" sheetId="4" r:id="rId3"/>
     <sheet name="RQ2-Bibliometric" sheetId="1" r:id="rId4"/>
     <sheet name="RQ4-Yu-Menzies Simulation" sheetId="5" r:id="rId5"/>
+    <sheet name="FitnessFunction" sheetId="6" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'RQ2-Bibliometric'!$A$1:$P$7</definedName>
@@ -44,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="647" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="699" uniqueCount="86">
   <si>
     <t>Dataset</t>
   </si>
@@ -214,16 +215,7 @@
     <t>TP FP TN FN</t>
   </si>
   <si>
-    <t>Time (min)</t>
-  </si>
-  <si>
-    <t>Nuestro mejor</t>
-  </si>
-  <si>
     <t>Algorithm</t>
-  </si>
-  <si>
-    <t>Ours</t>
   </si>
   <si>
     <t>FAST2</t>
@@ -240,6 +232,78 @@
   <si>
     <t>Default</t>
   </si>
+  <si>
+    <t>FAST2 Time (min)</t>
+  </si>
+  <si>
+    <t>IRECS Time (min)</t>
+  </si>
+  <si>
+    <t>33,4 h</t>
+  </si>
+  <si>
+    <t>7,7 h</t>
+  </si>
+  <si>
+    <t>28,8 h</t>
+  </si>
+  <si>
+    <t>79 s</t>
+  </si>
+  <si>
+    <t>IRECS</t>
+  </si>
+  <si>
+    <t>fitnessStrategy</t>
+  </si>
+  <si>
+    <t>balancedAcc_mean</t>
+  </si>
+  <si>
+    <t>balancedAcc_std</t>
+  </si>
+  <si>
+    <t>accuracy_mean</t>
+  </si>
+  <si>
+    <t>accuracy_std</t>
+  </si>
+  <si>
+    <t>precision_mean</t>
+  </si>
+  <si>
+    <t>precision_std</t>
+  </si>
+  <si>
+    <t>recall_mean</t>
+  </si>
+  <si>
+    <t>recall_std</t>
+  </si>
+  <si>
+    <t>specificity_mean</t>
+  </si>
+  <si>
+    <t>specificity_std</t>
+  </si>
+  <si>
+    <t>lift</t>
+  </si>
+  <si>
+    <t>sup*conf</t>
+  </si>
+  <si>
+    <t>confidence</t>
+  </si>
+  <si>
+    <t>support</t>
+  </si>
+  <si>
+    <t>f1</t>
+  </si>
+  <si>
+    <t>irecs</t>
+  </si>
 </sst>
 </file>
 
@@ -248,7 +312,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="11">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -290,6 +354,28 @@
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -367,7 +453,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="17">
     <border>
       <left/>
       <right/>
@@ -469,11 +555,97 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="67">
+  <cellXfs count="83">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -530,7 +702,6 @@
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -555,6 +726,23 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2760,7 +2948,7 @@
       </c>
       <c r="O4" s="30"/>
     </row>
-    <row r="5" spans="1:15">
+    <row r="5" spans="1:15" ht="12.75">
       <c r="A5" s="1" t="s">
         <v>30</v>
       </c>
@@ -2895,7 +3083,7 @@
       </c>
       <c r="O7" s="30"/>
     </row>
-    <row r="8" spans="1:15">
+    <row r="8" spans="1:15" ht="12.75">
       <c r="A8" s="1" t="s">
         <v>32</v>
       </c>
@@ -3030,7 +3218,7 @@
       </c>
       <c r="O10" s="30"/>
     </row>
-    <row r="11" spans="1:15">
+    <row r="11" spans="1:15" ht="12.75">
       <c r="A11" s="11" t="s">
         <v>20</v>
       </c>
@@ -3075,7 +3263,7 @@
       </c>
       <c r="O11" s="30"/>
     </row>
-    <row r="12" spans="1:15">
+    <row r="12" spans="1:15" ht="12.75">
       <c r="A12" s="1" t="s">
         <v>20</v>
       </c>
@@ -3120,7 +3308,7 @@
       </c>
       <c r="O12" s="30"/>
     </row>
-    <row r="13" spans="1:15">
+    <row r="13" spans="1:15" ht="12.75">
       <c r="A13" s="14" t="s">
         <v>20</v>
       </c>
@@ -3165,7 +3353,7 @@
       </c>
       <c r="O13" s="30"/>
     </row>
-    <row r="14" spans="1:15">
+    <row r="14" spans="1:15" ht="12.75">
       <c r="A14" s="11" t="s">
         <v>35</v>
       </c>
@@ -3210,7 +3398,7 @@
       </c>
       <c r="O14" s="30"/>
     </row>
-    <row r="15" spans="1:15">
+    <row r="15" spans="1:15" ht="12.75">
       <c r="A15" s="11" t="s">
         <v>35</v>
       </c>
@@ -3255,7 +3443,7 @@
       </c>
       <c r="O15" s="30"/>
     </row>
-    <row r="16" spans="1:15">
+    <row r="16" spans="1:15" ht="12.75">
       <c r="A16" s="11" t="s">
         <v>35</v>
       </c>
@@ -3300,13 +3488,13 @@
       </c>
       <c r="O16" s="30"/>
     </row>
-    <row r="17" spans="8:8">
+    <row r="17" spans="8:8" ht="12.75">
       <c r="H17" s="31"/>
     </row>
-    <row r="18" spans="8:8">
+    <row r="18" spans="8:8" ht="12.75">
       <c r="H18" s="31"/>
     </row>
-    <row r="19" spans="8:8">
+    <row r="19" spans="8:8" ht="12.75">
       <c r="H19" s="31"/>
     </row>
     <row r="39" spans="1:9" ht="12.75">
@@ -6189,7 +6377,7 @@
       </c>
       <c r="Q1" s="2"/>
     </row>
-    <row r="2" spans="1:17">
+    <row r="2" spans="1:17" ht="12.75">
       <c r="A2" s="1" t="s">
         <v>44</v>
       </c>
@@ -6241,7 +6429,7 @@
       </c>
       <c r="Q2" s="21"/>
     </row>
-    <row r="3" spans="1:17">
+    <row r="3" spans="1:17" ht="12.75">
       <c r="A3" s="1" t="s">
         <v>44</v>
       </c>
@@ -6293,7 +6481,7 @@
       </c>
       <c r="Q3" s="21"/>
     </row>
-    <row r="4" spans="1:17">
+    <row r="4" spans="1:17" ht="12.75">
       <c r="A4" s="1" t="s">
         <v>44</v>
       </c>
@@ -6345,7 +6533,7 @@
       </c>
       <c r="Q4" s="21"/>
     </row>
-    <row r="5" spans="1:17">
+    <row r="5" spans="1:17" ht="12.75">
       <c r="A5" s="1" t="s">
         <v>44</v>
       </c>
@@ -6397,7 +6585,7 @@
       </c>
       <c r="Q5" s="21"/>
     </row>
-    <row r="6" spans="1:17">
+    <row r="6" spans="1:17" ht="12.75">
       <c r="A6" s="1" t="s">
         <v>44</v>
       </c>
@@ -6449,7 +6637,7 @@
       </c>
       <c r="Q6" s="21"/>
     </row>
-    <row r="7" spans="1:17">
+    <row r="7" spans="1:17" ht="12.75">
       <c r="A7" s="1" t="s">
         <v>44</v>
       </c>
@@ -6501,7 +6689,7 @@
       </c>
       <c r="Q7" s="21"/>
     </row>
-    <row r="8" spans="1:17">
+    <row r="8" spans="1:17" ht="12.75">
       <c r="A8" s="11" t="s">
         <v>30</v>
       </c>
@@ -6553,7 +6741,7 @@
       </c>
       <c r="Q8" s="21"/>
     </row>
-    <row r="9" spans="1:17">
+    <row r="9" spans="1:17" ht="12.75">
       <c r="A9" s="1" t="s">
         <v>30</v>
       </c>
@@ -6605,7 +6793,7 @@
       </c>
       <c r="Q9" s="21"/>
     </row>
-    <row r="10" spans="1:17">
+    <row r="10" spans="1:17" ht="12.75">
       <c r="A10" s="1" t="s">
         <v>30</v>
       </c>
@@ -6657,7 +6845,7 @@
       </c>
       <c r="Q10" s="21"/>
     </row>
-    <row r="11" spans="1:17">
+    <row r="11" spans="1:17" ht="12.75">
       <c r="A11" s="1" t="s">
         <v>30</v>
       </c>
@@ -6709,7 +6897,7 @@
       </c>
       <c r="Q11" s="21"/>
     </row>
-    <row r="12" spans="1:17">
+    <row r="12" spans="1:17" ht="12.75">
       <c r="A12" s="1" t="s">
         <v>30</v>
       </c>
@@ -6761,7 +6949,7 @@
       </c>
       <c r="Q12" s="21"/>
     </row>
-    <row r="13" spans="1:17">
+    <row r="13" spans="1:17" ht="12.75">
       <c r="A13" s="14" t="s">
         <v>30</v>
       </c>
@@ -6813,7 +7001,7 @@
       </c>
       <c r="Q13" s="21"/>
     </row>
-    <row r="14" spans="1:17">
+    <row r="14" spans="1:17" ht="12.75">
       <c r="A14" s="1" t="s">
         <v>32</v>
       </c>
@@ -6865,7 +7053,7 @@
       </c>
       <c r="Q14" s="21"/>
     </row>
-    <row r="15" spans="1:17">
+    <row r="15" spans="1:17" ht="12.75">
       <c r="A15" s="1" t="s">
         <v>32</v>
       </c>
@@ -6917,7 +7105,7 @@
       </c>
       <c r="Q15" s="21"/>
     </row>
-    <row r="16" spans="1:17">
+    <row r="16" spans="1:17" ht="12.75">
       <c r="A16" s="1" t="s">
         <v>32</v>
       </c>
@@ -6969,7 +7157,7 @@
       </c>
       <c r="Q16" s="21"/>
     </row>
-    <row r="17" spans="1:17">
+    <row r="17" spans="1:17" ht="12.75">
       <c r="A17" s="1" t="s">
         <v>32</v>
       </c>
@@ -7021,7 +7209,7 @@
       </c>
       <c r="Q17" s="21"/>
     </row>
-    <row r="18" spans="1:17">
+    <row r="18" spans="1:17" ht="12.75">
       <c r="A18" s="1" t="s">
         <v>32</v>
       </c>
@@ -7073,7 +7261,7 @@
       </c>
       <c r="Q18" s="21"/>
     </row>
-    <row r="19" spans="1:17">
+    <row r="19" spans="1:17" ht="12.75">
       <c r="A19" s="1" t="s">
         <v>32</v>
       </c>
@@ -7125,7 +7313,7 @@
       </c>
       <c r="Q19" s="21"/>
     </row>
-    <row r="20" spans="1:17">
+    <row r="20" spans="1:17" ht="12.75">
       <c r="A20" s="11" t="s">
         <v>20</v>
       </c>
@@ -7177,7 +7365,7 @@
       </c>
       <c r="Q20" s="21"/>
     </row>
-    <row r="21" spans="1:17">
+    <row r="21" spans="1:17" ht="12.75">
       <c r="A21" s="1" t="s">
         <v>20</v>
       </c>
@@ -7229,7 +7417,7 @@
       </c>
       <c r="Q21" s="21"/>
     </row>
-    <row r="22" spans="1:17">
+    <row r="22" spans="1:17" ht="12.75">
       <c r="A22" s="1" t="s">
         <v>20</v>
       </c>
@@ -7281,7 +7469,7 @@
       </c>
       <c r="Q22" s="21"/>
     </row>
-    <row r="23" spans="1:17">
+    <row r="23" spans="1:17" ht="12.75">
       <c r="A23" s="1" t="s">
         <v>20</v>
       </c>
@@ -7333,7 +7521,7 @@
       </c>
       <c r="Q23" s="21"/>
     </row>
-    <row r="24" spans="1:17">
+    <row r="24" spans="1:17" ht="12.75">
       <c r="A24" s="1" t="s">
         <v>20</v>
       </c>
@@ -7385,7 +7573,7 @@
       </c>
       <c r="Q24" s="21"/>
     </row>
-    <row r="25" spans="1:17">
+    <row r="25" spans="1:17" ht="12.75">
       <c r="A25" s="1" t="s">
         <v>20</v>
       </c>
@@ -10694,7 +10882,7 @@
   <customSheetViews>
     <customSheetView guid="{7D8CF709-473A-4560-BB7E-E85A5A6A7688}" filter="1" showAutoFilter="1">
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-      <autoFilter ref="A1:P113" xr:uid="{F04BAF20-0E7F-4B0A-823C-3F3E00A68EAA}">
+      <autoFilter ref="A1:P113" xr:uid="{3993BCEA-4790-495C-9FE6-FE55F80F60AF}">
         <filterColumn colId="0">
           <filters>
             <filter val="AISE"/>
@@ -11086,7 +11274,7 @@
         <v>153.49219628333299</v>
       </c>
     </row>
-    <row r="13" spans="1:17">
+    <row r="13" spans="1:17" ht="12.75">
       <c r="B13" s="19"/>
       <c r="C13" s="19"/>
       <c r="D13" s="19"/>
@@ -11104,7 +11292,7 @@
       <c r="P13" s="19"/>
       <c r="Q13" s="19"/>
     </row>
-    <row r="14" spans="1:17">
+    <row r="14" spans="1:17" ht="12.75">
       <c r="B14" s="19"/>
       <c r="C14" s="19"/>
       <c r="D14" s="19"/>
@@ -11122,7 +11310,7 @@
       <c r="P14" s="19"/>
       <c r="Q14" s="19"/>
     </row>
-    <row r="15" spans="1:17">
+    <row r="15" spans="1:17" ht="12.75">
       <c r="B15" s="19"/>
       <c r="C15" s="19"/>
       <c r="D15" s="19"/>
@@ -11140,7 +11328,7 @@
       <c r="P15" s="19"/>
       <c r="Q15" s="19"/>
     </row>
-    <row r="16" spans="1:17">
+    <row r="16" spans="1:17" ht="12.75">
       <c r="B16" s="19"/>
       <c r="C16" s="19"/>
       <c r="D16" s="19"/>
@@ -11158,7 +11346,7 @@
       <c r="P16" s="19"/>
       <c r="Q16" s="19"/>
     </row>
-    <row r="17" spans="2:17">
+    <row r="17" spans="2:17" ht="12.75">
       <c r="B17" s="19"/>
       <c r="C17" s="19"/>
       <c r="D17" s="19"/>
@@ -11176,7 +11364,7 @@
       <c r="P17" s="19"/>
       <c r="Q17" s="19"/>
     </row>
-    <row r="18" spans="2:17">
+    <row r="18" spans="2:17" ht="12.75">
       <c r="B18" s="19"/>
       <c r="C18" s="19"/>
       <c r="D18" s="19"/>
@@ -11194,7 +11382,7 @@
       <c r="P18" s="19"/>
       <c r="Q18" s="19"/>
     </row>
-    <row r="19" spans="2:17">
+    <row r="19" spans="2:17" ht="12.75">
       <c r="B19" s="19"/>
       <c r="C19" s="19"/>
       <c r="D19" s="19"/>
@@ -11212,7 +11400,7 @@
       <c r="P19" s="19"/>
       <c r="Q19" s="19"/>
     </row>
-    <row r="20" spans="2:17">
+    <row r="20" spans="2:17" ht="12.75">
       <c r="B20" s="19"/>
       <c r="C20" s="19"/>
       <c r="D20" s="19"/>
@@ -11277,33 +11465,36 @@
         <v>55</v>
       </c>
       <c r="I1" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="J1" t="s">
+        <v>63</v>
+      </c>
+      <c r="K1" s="59" t="s">
+        <v>0</v>
+      </c>
+      <c r="L1" s="46" t="s">
         <v>56</v>
       </c>
-      <c r="K1" s="46" t="s">
-        <v>57</v>
-      </c>
-      <c r="L1" s="47" t="s">
-        <v>58</v>
-      </c>
-      <c r="M1" s="48" t="s">
+      <c r="M1" s="47" t="s">
         <v>10</v>
       </c>
-      <c r="N1" s="48" t="s">
+      <c r="N1" s="47" t="s">
         <v>11</v>
       </c>
-      <c r="O1" s="48" t="s">
+      <c r="O1" s="47" t="s">
         <v>12</v>
       </c>
-      <c r="P1" s="48" t="s">
+      <c r="P1" s="47" t="s">
         <v>13</v>
       </c>
-      <c r="Q1" s="48" t="s">
+      <c r="Q1" s="47" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="2" spans="1:17" ht="15.75" customHeight="1">
-      <c r="A2" s="19" t="s">
-        <v>44</v>
+      <c r="A2" s="69" t="s">
+        <v>15</v>
       </c>
       <c r="B2" s="1">
         <f t="shared" ref="B2:B5" si="0">(E2+F2)/2</f>
@@ -11325,30 +11516,36 @@
         <v>6.7524115755627001E-2</v>
       </c>
       <c r="H2" s="2"/>
-      <c r="K2" s="64" t="s">
-        <v>44</v>
-      </c>
-      <c r="L2" s="49" t="s">
-        <v>59</v>
-      </c>
-      <c r="M2" s="50">
+      <c r="I2" t="s">
+        <v>64</v>
+      </c>
+      <c r="J2">
+        <v>55</v>
+      </c>
+      <c r="K2" s="67" t="s">
+        <v>15</v>
+      </c>
+      <c r="L2" s="66" t="s">
+        <v>68</v>
+      </c>
+      <c r="M2" s="49">
         <v>0.87129900000000005</v>
       </c>
-      <c r="N2" s="51">
+      <c r="N2" s="50">
         <v>0.78683800000000004</v>
       </c>
-      <c r="O2" s="51">
+      <c r="O2" s="50">
         <v>5.9458999999999998E-2</v>
       </c>
-      <c r="P2" s="51">
+      <c r="P2" s="50">
         <v>0.95797900000000002</v>
       </c>
-      <c r="Q2" s="51">
+      <c r="Q2" s="50">
         <v>0.78461899999999996</v>
       </c>
     </row>
     <row r="3" spans="1:17" ht="15.75" customHeight="1">
-      <c r="A3" s="52" t="s">
+      <c r="A3" s="51" t="s">
         <v>30</v>
       </c>
       <c r="B3" s="14">
@@ -11371,24 +11568,30 @@
         <v>8.1784386617100302E-2</v>
       </c>
       <c r="H3" s="3"/>
-      <c r="K3" s="63"/>
-      <c r="L3" s="49" t="s">
-        <v>60</v>
-      </c>
-      <c r="M3" s="53">
+      <c r="I3" t="s">
+        <v>65</v>
+      </c>
+      <c r="J3">
+        <v>49</v>
+      </c>
+      <c r="K3" s="62"/>
+      <c r="L3" s="48" t="s">
+        <v>57</v>
+      </c>
+      <c r="M3" s="52">
         <f>(P3+Q3)/2</f>
         <v>0.73083685380088348</v>
       </c>
-      <c r="N3" s="53">
+      <c r="N3" s="52">
         <v>0.783015338570894</v>
       </c>
-      <c r="O3" s="53">
+      <c r="O3" s="52">
         <v>3.5532994923857801E-2</v>
       </c>
-      <c r="P3" s="53">
+      <c r="P3" s="52">
         <v>0.67741935483870896</v>
       </c>
-      <c r="Q3" s="53">
+      <c r="Q3" s="52">
         <v>0.78425435276305799</v>
       </c>
     </row>
@@ -11416,30 +11619,36 @@
         <v>4.08163265306122E-2</v>
       </c>
       <c r="H4" s="2"/>
-      <c r="K4" s="64" t="s">
+      <c r="I4" t="s">
+        <v>66</v>
+      </c>
+      <c r="J4">
+        <v>51</v>
+      </c>
+      <c r="K4" s="63" t="s">
         <v>30</v>
       </c>
-      <c r="L4" s="49" t="s">
-        <v>59</v>
-      </c>
-      <c r="M4" s="51">
+      <c r="L4" s="66" t="s">
+        <v>68</v>
+      </c>
+      <c r="M4" s="50">
         <v>0.735286</v>
       </c>
-      <c r="N4" s="51">
+      <c r="N4" s="50">
         <v>0.64411300000000005</v>
       </c>
-      <c r="O4" s="51">
+      <c r="O4" s="50">
         <v>6.1062999999999999E-2</v>
       </c>
-      <c r="P4" s="51">
+      <c r="P4" s="50">
         <v>0.83152199999999998</v>
       </c>
-      <c r="Q4" s="51">
+      <c r="Q4" s="50">
         <v>0.63905000000000001</v>
       </c>
     </row>
-    <row r="5" spans="1:17">
-      <c r="A5" s="54" t="s">
+    <row r="5" spans="1:17" ht="12.75">
+      <c r="A5" s="53" t="s">
         <v>20</v>
       </c>
       <c r="B5" s="11">
@@ -11462,30 +11671,36 @@
         <v>0</v>
       </c>
       <c r="H5" s="11" t="s">
-        <v>61</v>
-      </c>
-      <c r="K5" s="63"/>
-      <c r="L5" s="49" t="s">
-        <v>60</v>
-      </c>
-      <c r="M5" s="53">
+        <v>58</v>
+      </c>
+      <c r="I5" t="s">
+        <v>67</v>
+      </c>
+      <c r="J5">
+        <v>2.1329530170000002</v>
+      </c>
+      <c r="K5" s="62"/>
+      <c r="L5" s="48" t="s">
+        <v>57</v>
+      </c>
+      <c r="M5" s="52">
         <f>(P5+Q5)/2</f>
         <v>0.64787722317842755</v>
       </c>
-      <c r="N5" s="53">
+      <c r="N5" s="52">
         <v>0.517578125</v>
       </c>
-      <c r="O5" s="53">
+      <c r="O5" s="52">
         <v>4.31372549019607E-2</v>
       </c>
-      <c r="P5" s="53">
+      <c r="P5" s="52">
         <v>0.78571428571428503</v>
       </c>
-      <c r="Q5" s="53">
+      <c r="Q5" s="52">
         <v>0.51004016064256996</v>
       </c>
     </row>
-    <row r="6" spans="1:17">
+    <row r="6" spans="1:17" ht="12.75">
       <c r="A6" s="1" t="s">
         <v>21</v>
       </c>
@@ -11505,99 +11720,102 @@
         <v>0.34735706580366699</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="K6" s="64" t="s">
+        <v>60</v>
+      </c>
+      <c r="J6">
+        <v>143.53842510000001</v>
+      </c>
+      <c r="K6" s="63" t="s">
         <v>32</v>
       </c>
-      <c r="L6" s="49" t="s">
-        <v>59</v>
-      </c>
-      <c r="M6" s="51">
+      <c r="L6" s="66" t="s">
+        <v>68</v>
+      </c>
+      <c r="M6" s="50">
         <v>0.81994599999999995</v>
       </c>
-      <c r="N6" s="55">
+      <c r="N6" s="54">
         <v>0.67952000000000001</v>
       </c>
-      <c r="O6" s="51">
+      <c r="O6" s="50">
         <v>2.6717999999999999E-2</v>
       </c>
-      <c r="P6" s="51">
+      <c r="P6" s="50">
         <v>0.96290299999999995</v>
       </c>
-      <c r="Q6" s="55">
+      <c r="Q6" s="54">
         <v>0.67698800000000003</v>
       </c>
     </row>
-    <row r="7" spans="1:17">
-      <c r="K7" s="63"/>
-      <c r="L7" s="49" t="s">
-        <v>60</v>
-      </c>
-      <c r="M7" s="53">
+    <row r="7" spans="1:17" ht="12.75">
+      <c r="K7" s="62"/>
+      <c r="L7" s="48" t="s">
+        <v>57</v>
+      </c>
+      <c r="M7" s="52">
         <f>(P7+Q7)/2</f>
         <v>0.66723545174174603</v>
       </c>
-      <c r="N7" s="56">
+      <c r="N7" s="55">
         <v>0.75392670157067998</v>
       </c>
-      <c r="O7" s="53">
+      <c r="O7" s="52">
         <v>2.11538461538461E-2</v>
       </c>
-      <c r="P7" s="53">
+      <c r="P7" s="52">
         <v>0.57894736842105199</v>
       </c>
-      <c r="Q7" s="56">
+      <c r="Q7" s="55">
         <v>0.75552353506243997</v>
       </c>
     </row>
-    <row r="8" spans="1:17">
+    <row r="8" spans="1:17" ht="12.75">
       <c r="A8" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="B8" s="57">
+      <c r="B8" s="56">
         <v>0.5</v>
       </c>
-      <c r="C8" s="57">
+      <c r="C8" s="56">
         <v>0.58612440241168129</v>
       </c>
-      <c r="D8" s="57">
+      <c r="D8" s="56">
         <v>7.4525388725023303E-2</v>
       </c>
-      <c r="E8" s="57">
+      <c r="E8" s="56">
         <v>0.35</v>
       </c>
-      <c r="F8" s="57">
+      <c r="F8" s="56">
         <v>0.65</v>
       </c>
-      <c r="K8" s="65" t="s">
+      <c r="K8" s="64" t="s">
         <v>20</v>
       </c>
-      <c r="L8" s="49" t="s">
-        <v>59</v>
-      </c>
-      <c r="M8" s="51">
+      <c r="L8" s="66" t="s">
+        <v>68</v>
+      </c>
+      <c r="M8" s="50">
         <v>0.70348299999999997</v>
       </c>
-      <c r="N8" s="55">
+      <c r="N8" s="54">
         <v>0.79776499999999995</v>
       </c>
-      <c r="O8" s="51">
+      <c r="O8" s="50">
         <v>8.5141999999999995E-2</v>
       </c>
-      <c r="P8" s="51">
+      <c r="P8" s="50">
         <v>0.60357099999999997</v>
       </c>
-      <c r="Q8" s="55">
+      <c r="Q8" s="54">
         <v>0.80339400000000005</v>
       </c>
     </row>
     <row r="9" spans="1:17" ht="15.75" customHeight="1">
       <c r="A9" s="1" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="B9" s="27">
         <v>0.55059205570696301</v>
@@ -11614,432 +11832,432 @@
       <c r="F9" s="3">
         <v>0.94098662978331005</v>
       </c>
-      <c r="K9" s="63"/>
-      <c r="L9" s="49" t="s">
-        <v>60</v>
-      </c>
-      <c r="M9" s="58">
+      <c r="K9" s="62"/>
+      <c r="L9" s="48" t="s">
+        <v>57</v>
+      </c>
+      <c r="M9" s="57">
         <f>(P9+Q9)/2</f>
         <v>0.5</v>
       </c>
-      <c r="N9" s="59">
+      <c r="N9" s="58">
         <v>0.97080291970802901</v>
       </c>
-      <c r="O9" s="58">
+      <c r="O9" s="57">
         <v>0</v>
       </c>
-      <c r="P9" s="58">
+      <c r="P9" s="57">
         <v>0</v>
       </c>
-      <c r="Q9" s="59">
+      <c r="Q9" s="58">
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:17">
-      <c r="K10" s="66" t="s">
+    <row r="10" spans="1:17" ht="12.75">
+      <c r="K10" s="65" t="s">
         <v>21</v>
       </c>
-      <c r="L10" s="49" t="s">
-        <v>59</v>
-      </c>
-      <c r="M10" s="51">
+      <c r="L10" s="66" t="s">
+        <v>68</v>
+      </c>
+      <c r="M10" s="50">
         <v>0.49827100000000002</v>
       </c>
-      <c r="N10" s="51">
+      <c r="N10" s="50">
         <v>0.24202299999999999</v>
       </c>
-      <c r="O10" s="55">
+      <c r="O10" s="54">
         <v>0.20169999999999999</v>
       </c>
-      <c r="P10" s="51">
+      <c r="P10" s="50">
         <v>0.94458399999999998</v>
       </c>
-      <c r="Q10" s="51">
+      <c r="Q10" s="50">
         <v>5.1957000000000003E-2</v>
       </c>
     </row>
-    <row r="11" spans="1:17">
-      <c r="K11" s="63"/>
-      <c r="L11" s="49" t="s">
-        <v>60</v>
-      </c>
-      <c r="M11" s="53">
+    <row r="11" spans="1:17" ht="12.75">
+      <c r="K11" s="62"/>
+      <c r="L11" s="48" t="s">
+        <v>57</v>
+      </c>
+      <c r="M11" s="52">
         <v>0.43077956989247301</v>
       </c>
-      <c r="N11" s="53">
+      <c r="N11" s="52">
         <v>0.22976554536187499</v>
       </c>
-      <c r="O11" s="56">
+      <c r="O11" s="55">
         <v>0.71148989898989901</v>
       </c>
-      <c r="P11" s="53">
+      <c r="P11" s="52">
         <v>0.354849726775956</v>
       </c>
-      <c r="Q11" s="53">
+      <c r="Q11" s="52">
         <v>0.34735706580366699</v>
       </c>
     </row>
-    <row r="14" spans="1:17">
-      <c r="K14" s="60" t="s">
+    <row r="14" spans="1:17" ht="12.75">
+      <c r="K14" s="59" t="s">
         <v>0</v>
       </c>
-      <c r="L14" s="60" t="s">
-        <v>58</v>
-      </c>
-      <c r="M14" s="60" t="s">
+      <c r="L14" s="59" t="s">
+        <v>56</v>
+      </c>
+      <c r="M14" s="59" t="s">
         <v>10</v>
       </c>
-      <c r="N14" s="60" t="s">
+      <c r="N14" s="59" t="s">
         <v>11</v>
       </c>
-      <c r="O14" s="60" t="s">
+      <c r="O14" s="59" t="s">
         <v>12</v>
       </c>
-      <c r="P14" s="60" t="s">
+      <c r="P14" s="59" t="s">
         <v>13</v>
       </c>
-      <c r="Q14" s="60" t="s">
+      <c r="Q14" s="59" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="15" spans="1:17">
-      <c r="K15" s="62" t="s">
-        <v>44</v>
-      </c>
-      <c r="L15" s="58" t="s">
-        <v>59</v>
-      </c>
-      <c r="M15" s="60">
+    <row r="15" spans="1:17" ht="12.75">
+      <c r="K15" s="68" t="s">
+        <v>15</v>
+      </c>
+      <c r="L15" s="70" t="s">
+        <v>68</v>
+      </c>
+      <c r="M15" s="59">
         <v>0.87129900000000005</v>
       </c>
-      <c r="N15" s="60">
+      <c r="N15" s="59">
         <v>0.78683800000000004</v>
       </c>
-      <c r="O15" s="60">
+      <c r="O15" s="59">
         <v>5.9458999999999998E-2</v>
       </c>
-      <c r="P15" s="60">
+      <c r="P15" s="59">
         <v>0.95797900000000002</v>
       </c>
-      <c r="Q15" s="60">
+      <c r="Q15" s="59">
         <v>0.78461899999999996</v>
       </c>
     </row>
-    <row r="16" spans="1:17">
+    <row r="16" spans="1:17" ht="12.75">
       <c r="H16" s="1"/>
-      <c r="K16" s="63"/>
-      <c r="L16" s="58" t="s">
-        <v>60</v>
-      </c>
-      <c r="M16" s="58">
+      <c r="K16" s="62"/>
+      <c r="L16" s="57" t="s">
+        <v>57</v>
+      </c>
+      <c r="M16" s="57">
         <v>0.73083685380088348</v>
       </c>
-      <c r="N16" s="58">
+      <c r="N16" s="57">
         <v>0.783015338570894</v>
       </c>
-      <c r="O16" s="58">
+      <c r="O16" s="57">
         <v>3.5532994923857801E-2</v>
       </c>
-      <c r="P16" s="58">
+      <c r="P16" s="57">
         <v>0.67741935483870896</v>
       </c>
-      <c r="Q16" s="58">
+      <c r="Q16" s="57">
         <v>0.78425435276305799</v>
       </c>
     </row>
-    <row r="17" spans="8:17">
+    <row r="17" spans="8:17" ht="12.75">
       <c r="H17" s="1"/>
-      <c r="K17" s="58"/>
-      <c r="L17" s="58"/>
-      <c r="M17" s="58">
+      <c r="K17" s="57"/>
+      <c r="L17" s="57"/>
+      <c r="M17" s="57">
         <f t="shared" ref="M17:Q17" si="1">M15-M16</f>
         <v>0.14046214619911657</v>
       </c>
-      <c r="N17" s="58">
+      <c r="N17" s="57">
         <f t="shared" si="1"/>
         <v>3.8226614291060335E-3</v>
       </c>
-      <c r="O17" s="58">
+      <c r="O17" s="57">
         <f t="shared" si="1"/>
         <v>2.3926005076142197E-2</v>
       </c>
-      <c r="P17" s="58">
+      <c r="P17" s="57">
         <f t="shared" si="1"/>
         <v>0.28055964516129106</v>
       </c>
-      <c r="Q17" s="58">
+      <c r="Q17" s="57">
         <f t="shared" si="1"/>
         <v>3.6464723694196177E-4</v>
       </c>
     </row>
-    <row r="18" spans="8:17">
-      <c r="K18" s="62" t="s">
+    <row r="18" spans="8:17" ht="12.75">
+      <c r="K18" s="61" t="s">
         <v>30</v>
       </c>
-      <c r="L18" s="58" t="s">
-        <v>59</v>
-      </c>
-      <c r="M18" s="60">
+      <c r="L18" s="70" t="s">
+        <v>68</v>
+      </c>
+      <c r="M18" s="59">
         <v>0.735286</v>
       </c>
-      <c r="N18" s="60">
+      <c r="N18" s="59">
         <v>0.64411300000000005</v>
       </c>
-      <c r="O18" s="60">
+      <c r="O18" s="59">
         <v>6.1062999999999999E-2</v>
       </c>
-      <c r="P18" s="60">
+      <c r="P18" s="59">
         <v>0.83152199999999998</v>
       </c>
-      <c r="Q18" s="60">
+      <c r="Q18" s="59">
         <v>0.63905000000000001</v>
       </c>
     </row>
-    <row r="19" spans="8:17">
-      <c r="K19" s="63"/>
-      <c r="L19" s="58" t="s">
-        <v>60</v>
-      </c>
-      <c r="M19" s="58">
+    <row r="19" spans="8:17" ht="12.75">
+      <c r="K19" s="62"/>
+      <c r="L19" s="57" t="s">
+        <v>57</v>
+      </c>
+      <c r="M19" s="57">
         <v>0.64787722317842755</v>
       </c>
-      <c r="N19" s="58">
+      <c r="N19" s="57">
         <v>0.517578125</v>
       </c>
-      <c r="O19" s="58">
+      <c r="O19" s="57">
         <v>4.31372549019607E-2</v>
       </c>
-      <c r="P19" s="58">
+      <c r="P19" s="57">
         <v>0.78571428571428503</v>
       </c>
-      <c r="Q19" s="58">
+      <c r="Q19" s="57">
         <v>0.51004016064256996</v>
       </c>
     </row>
-    <row r="20" spans="8:17">
-      <c r="K20" s="58"/>
-      <c r="L20" s="58"/>
-      <c r="M20" s="58">
+    <row r="20" spans="8:17" ht="12.75">
+      <c r="K20" s="57"/>
+      <c r="L20" s="57"/>
+      <c r="M20" s="57">
         <f t="shared" ref="M20:Q20" si="2">M18-M19</f>
         <v>8.7408776821572443E-2</v>
       </c>
-      <c r="N20" s="58">
+      <c r="N20" s="57">
         <f t="shared" si="2"/>
         <v>0.12653487500000005</v>
       </c>
-      <c r="O20" s="58">
+      <c r="O20" s="57">
         <f t="shared" si="2"/>
         <v>1.7925745098039299E-2</v>
       </c>
-      <c r="P20" s="58">
+      <c r="P20" s="57">
         <f t="shared" si="2"/>
         <v>4.5807714285714951E-2</v>
       </c>
-      <c r="Q20" s="58">
+      <c r="Q20" s="57">
         <f t="shared" si="2"/>
         <v>0.12900983935743005</v>
       </c>
     </row>
-    <row r="21" spans="8:17">
-      <c r="K21" s="62" t="s">
+    <row r="21" spans="8:17" ht="12.75">
+      <c r="K21" s="61" t="s">
         <v>32</v>
       </c>
-      <c r="L21" s="58" t="s">
-        <v>59</v>
-      </c>
-      <c r="M21" s="60">
+      <c r="L21" s="70" t="s">
+        <v>68</v>
+      </c>
+      <c r="M21" s="59">
         <v>0.81994599999999995</v>
       </c>
-      <c r="N21" s="58">
+      <c r="N21" s="57">
         <v>0.67952000000000001</v>
       </c>
-      <c r="O21" s="60">
+      <c r="O21" s="59">
         <v>2.6717999999999999E-2</v>
       </c>
-      <c r="P21" s="60">
+      <c r="P21" s="59">
         <v>0.96290299999999995</v>
       </c>
-      <c r="Q21" s="58">
+      <c r="Q21" s="57">
         <v>0.67698800000000003</v>
       </c>
     </row>
-    <row r="22" spans="8:17">
-      <c r="K22" s="63"/>
-      <c r="L22" s="58" t="s">
-        <v>60</v>
-      </c>
-      <c r="M22" s="58">
+    <row r="22" spans="8:17" ht="12.75">
+      <c r="K22" s="62"/>
+      <c r="L22" s="57" t="s">
+        <v>57</v>
+      </c>
+      <c r="M22" s="57">
         <v>0.66723545174174603</v>
       </c>
-      <c r="N22" s="60">
+      <c r="N22" s="59">
         <v>0.75392670157067998</v>
       </c>
-      <c r="O22" s="58">
+      <c r="O22" s="57">
         <v>2.11538461538461E-2</v>
       </c>
-      <c r="P22" s="58">
+      <c r="P22" s="57">
         <v>0.57894736842105199</v>
       </c>
-      <c r="Q22" s="60">
+      <c r="Q22" s="59">
         <v>0.75552353506243997</v>
       </c>
     </row>
-    <row r="23" spans="8:17">
-      <c r="K23" s="58"/>
-      <c r="L23" s="58"/>
-      <c r="M23" s="58">
+    <row r="23" spans="8:17" ht="12.75">
+      <c r="K23" s="57"/>
+      <c r="L23" s="57"/>
+      <c r="M23" s="57">
         <f t="shared" ref="M23:Q23" si="3">M21-M22</f>
         <v>0.15271054825825392</v>
       </c>
-      <c r="N23" s="58">
+      <c r="N23" s="57">
         <f t="shared" si="3"/>
         <v>-7.4406701570679967E-2</v>
       </c>
-      <c r="O23" s="58">
+      <c r="O23" s="57">
         <f t="shared" si="3"/>
         <v>5.5641538461538992E-3</v>
       </c>
-      <c r="P23" s="58">
+      <c r="P23" s="57">
         <f t="shared" si="3"/>
         <v>0.38395563157894796</v>
       </c>
-      <c r="Q23" s="58">
+      <c r="Q23" s="57">
         <f t="shared" si="3"/>
         <v>-7.8535535062439932E-2</v>
       </c>
     </row>
-    <row r="24" spans="8:17">
-      <c r="K24" s="62" t="s">
+    <row r="24" spans="8:17" ht="12.75">
+      <c r="K24" s="61" t="s">
         <v>20</v>
       </c>
-      <c r="L24" s="58" t="s">
-        <v>59</v>
-      </c>
-      <c r="M24" s="60">
+      <c r="L24" s="70" t="s">
+        <v>68</v>
+      </c>
+      <c r="M24" s="59">
         <v>0.70348299999999997</v>
       </c>
-      <c r="N24" s="58">
+      <c r="N24" s="57">
         <v>0.79776499999999995</v>
       </c>
-      <c r="O24" s="60">
+      <c r="O24" s="59">
         <v>8.5141999999999995E-2</v>
       </c>
-      <c r="P24" s="60">
+      <c r="P24" s="59">
         <v>0.60357099999999997</v>
       </c>
-      <c r="Q24" s="58">
+      <c r="Q24" s="57">
         <v>0.80339400000000005</v>
       </c>
     </row>
-    <row r="25" spans="8:17">
-      <c r="K25" s="63"/>
-      <c r="L25" s="58" t="s">
-        <v>60</v>
-      </c>
-      <c r="M25" s="58">
+    <row r="25" spans="8:17" ht="12.75">
+      <c r="K25" s="62"/>
+      <c r="L25" s="57" t="s">
+        <v>57</v>
+      </c>
+      <c r="M25" s="57">
         <v>0.5</v>
       </c>
-      <c r="N25" s="60">
+      <c r="N25" s="59">
         <v>0.97080291970802901</v>
       </c>
-      <c r="O25" s="58">
+      <c r="O25" s="57">
         <v>0</v>
       </c>
-      <c r="P25" s="58">
+      <c r="P25" s="57">
         <v>0</v>
       </c>
-      <c r="Q25" s="60">
+      <c r="Q25" s="59">
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="8:17">
-      <c r="K26" s="58"/>
-      <c r="L26" s="58"/>
-      <c r="M26" s="58">
+    <row r="26" spans="8:17" ht="12.75">
+      <c r="K26" s="57"/>
+      <c r="L26" s="57"/>
+      <c r="M26" s="57">
         <f t="shared" ref="M26:Q26" si="4">M24-M25</f>
         <v>0.20348299999999997</v>
       </c>
-      <c r="N26" s="58">
+      <c r="N26" s="57">
         <f t="shared" si="4"/>
         <v>-0.17303791970802906</v>
       </c>
-      <c r="O26" s="58">
+      <c r="O26" s="57">
         <f t="shared" si="4"/>
         <v>8.5141999999999995E-2</v>
       </c>
-      <c r="P26" s="58">
+      <c r="P26" s="57">
         <f t="shared" si="4"/>
         <v>0.60357099999999997</v>
       </c>
-      <c r="Q26" s="58">
+      <c r="Q26" s="57">
         <f t="shared" si="4"/>
         <v>-0.19660599999999995</v>
       </c>
     </row>
-    <row r="27" spans="8:17">
-      <c r="K27" s="62" t="s">
+    <row r="27" spans="8:17" ht="12.75">
+      <c r="K27" s="61" t="s">
         <v>21</v>
       </c>
-      <c r="L27" s="58" t="s">
-        <v>59</v>
-      </c>
-      <c r="M27" s="60">
+      <c r="L27" s="70" t="s">
+        <v>68</v>
+      </c>
+      <c r="M27" s="59">
         <v>0.49827100000000002</v>
       </c>
-      <c r="N27" s="60">
+      <c r="N27" s="59">
         <v>0.24202299999999999</v>
       </c>
-      <c r="O27" s="58">
+      <c r="O27" s="57">
         <v>0.20169999999999999</v>
       </c>
-      <c r="P27" s="60">
+      <c r="P27" s="59">
         <v>0.94458399999999998</v>
       </c>
-      <c r="Q27" s="60">
+      <c r="Q27" s="59">
         <v>5.1957000000000003E-2</v>
       </c>
     </row>
-    <row r="28" spans="8:17">
-      <c r="K28" s="63"/>
-      <c r="L28" s="58" t="s">
-        <v>60</v>
-      </c>
-      <c r="M28" s="58">
+    <row r="28" spans="8:17" ht="12.75">
+      <c r="K28" s="62"/>
+      <c r="L28" s="57" t="s">
+        <v>57</v>
+      </c>
+      <c r="M28" s="57">
         <v>0.43077956989247301</v>
       </c>
-      <c r="N28" s="58">
+      <c r="N28" s="57">
         <v>0.22976554536187499</v>
       </c>
-      <c r="O28" s="60">
+      <c r="O28" s="59">
         <v>0.71148989898989901</v>
       </c>
-      <c r="P28" s="58">
+      <c r="P28" s="57">
         <v>0.354849726775956</v>
       </c>
-      <c r="Q28" s="58">
+      <c r="Q28" s="57">
         <v>0.34735706580366699</v>
       </c>
     </row>
-    <row r="29" spans="8:17">
+    <row r="29" spans="8:17" ht="12.75">
       <c r="K29" s="1"/>
       <c r="L29" s="1"/>
-      <c r="M29" s="58">
+      <c r="M29" s="57">
         <f t="shared" ref="M29:Q29" si="5">M27-M28</f>
         <v>6.7491430107527006E-2</v>
       </c>
-      <c r="N29" s="58">
+      <c r="N29" s="57">
         <f t="shared" si="5"/>
         <v>1.2257454638124998E-2</v>
       </c>
-      <c r="O29" s="61">
+      <c r="O29" s="60">
         <f t="shared" si="5"/>
         <v>-0.50978989898989902</v>
       </c>
-      <c r="P29" s="58">
+      <c r="P29" s="57">
         <f t="shared" si="5"/>
         <v>0.58973427322404404</v>
       </c>
-      <c r="Q29" s="58">
+      <c r="Q29" s="57">
         <f t="shared" si="5"/>
         <v>-0.29540006580366696</v>
       </c>
@@ -12080,4 +12298,1142 @@
     <tablePart r:id="rId3"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33AF8091-6052-47A2-AE0B-B3D7862DD150}">
+  <dimension ref="A1:L31"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75"/>
+  <sheetData>
+    <row r="1" spans="1:12">
+      <c r="A1" s="78" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="78" t="s">
+        <v>69</v>
+      </c>
+      <c r="C1" s="71" t="s">
+        <v>70</v>
+      </c>
+      <c r="D1" s="71" t="s">
+        <v>71</v>
+      </c>
+      <c r="E1" s="71" t="s">
+        <v>72</v>
+      </c>
+      <c r="F1" s="71" t="s">
+        <v>73</v>
+      </c>
+      <c r="G1" s="71" t="s">
+        <v>74</v>
+      </c>
+      <c r="H1" s="71" t="s">
+        <v>75</v>
+      </c>
+      <c r="I1" s="71" t="s">
+        <v>76</v>
+      </c>
+      <c r="J1" s="71" t="s">
+        <v>77</v>
+      </c>
+      <c r="K1" s="71" t="s">
+        <v>78</v>
+      </c>
+      <c r="L1" s="71" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12">
+      <c r="A2" s="79" t="s">
+        <v>15</v>
+      </c>
+      <c r="B2" s="82" t="s">
+        <v>85</v>
+      </c>
+      <c r="C2" s="72">
+        <v>0.73211944760000003</v>
+      </c>
+      <c r="D2" s="72">
+        <v>0.11802258359999999</v>
+      </c>
+      <c r="E2" s="72">
+        <v>0.88135680059999999</v>
+      </c>
+      <c r="F2" s="72">
+        <v>7.2815491910000002E-2</v>
+      </c>
+      <c r="G2" s="72">
+        <v>4.986476904E-2</v>
+      </c>
+      <c r="H2" s="72">
+        <v>2.664941622E-2</v>
+      </c>
+      <c r="I2" s="72">
+        <v>0.579245283</v>
+      </c>
+      <c r="J2" s="72">
+        <v>0.30821460420000002</v>
+      </c>
+      <c r="K2" s="72">
+        <v>0.88499361210000005</v>
+      </c>
+      <c r="L2" s="73">
+        <v>7.7210030269999994E-2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12">
+      <c r="A3" s="80"/>
+      <c r="B3" s="80" t="s">
+        <v>80</v>
+      </c>
+      <c r="C3" s="74">
+        <v>0.51596463250000002</v>
+      </c>
+      <c r="D3" s="74">
+        <v>2.6980865359999998E-2</v>
+      </c>
+      <c r="E3" s="74">
+        <v>0.98649978739999999</v>
+      </c>
+      <c r="F3" s="74">
+        <v>2.4364026519999998E-3</v>
+      </c>
+      <c r="G3" s="74">
+        <v>6.7108714659999999E-2</v>
+      </c>
+      <c r="H3" s="74">
+        <v>7.355770532E-2</v>
+      </c>
+      <c r="I3" s="74">
+        <v>3.3962264149999997E-2</v>
+      </c>
+      <c r="J3" s="74">
+        <v>5.69868241E-2</v>
+      </c>
+      <c r="K3" s="74">
+        <v>0.99796700090000001</v>
+      </c>
+      <c r="L3" s="75">
+        <v>3.1252832609999998E-3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12">
+      <c r="A4" s="80"/>
+      <c r="B4" s="80" t="s">
+        <v>81</v>
+      </c>
+      <c r="C4" s="74">
+        <v>0.5</v>
+      </c>
+      <c r="D4" s="74">
+        <v>0</v>
+      </c>
+      <c r="E4" s="74">
+        <v>0.98810458970000004</v>
+      </c>
+      <c r="F4" s="74">
+        <v>0</v>
+      </c>
+      <c r="G4" s="74">
+        <v>0</v>
+      </c>
+      <c r="H4" s="74">
+        <v>0</v>
+      </c>
+      <c r="I4" s="74">
+        <v>0</v>
+      </c>
+      <c r="J4" s="74">
+        <v>0</v>
+      </c>
+      <c r="K4" s="74">
+        <v>1</v>
+      </c>
+      <c r="L4" s="75">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12">
+      <c r="A5" s="80"/>
+      <c r="B5" s="80" t="s">
+        <v>82</v>
+      </c>
+      <c r="C5" s="74">
+        <v>0.50137533970000003</v>
+      </c>
+      <c r="D5" s="74">
+        <v>4.3492059539999997E-3</v>
+      </c>
+      <c r="E5" s="74">
+        <v>0.98805969630000001</v>
+      </c>
+      <c r="F5" s="74">
+        <v>1.419653271E-4</v>
+      </c>
+      <c r="G5" s="74">
+        <v>1.4999999999999999E-2</v>
+      </c>
+      <c r="H5" s="74">
+        <v>4.7434164899999999E-2</v>
+      </c>
+      <c r="I5" s="74">
+        <v>2.8301886789999999E-3</v>
+      </c>
+      <c r="J5" s="74">
+        <v>8.9498424340000004E-3</v>
+      </c>
+      <c r="K5" s="74">
+        <v>0.9999204907</v>
+      </c>
+      <c r="L5" s="75">
+        <v>2.5143052730000002E-4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12">
+      <c r="A6" s="80"/>
+      <c r="B6" s="80" t="s">
+        <v>83</v>
+      </c>
+      <c r="C6" s="74">
+        <v>0.5</v>
+      </c>
+      <c r="D6" s="74">
+        <v>0</v>
+      </c>
+      <c r="E6" s="74">
+        <v>0.98810458970000004</v>
+      </c>
+      <c r="F6" s="74">
+        <v>0</v>
+      </c>
+      <c r="G6" s="74">
+        <v>0</v>
+      </c>
+      <c r="H6" s="74">
+        <v>0</v>
+      </c>
+      <c r="I6" s="74">
+        <v>0</v>
+      </c>
+      <c r="J6" s="74">
+        <v>0</v>
+      </c>
+      <c r="K6" s="74">
+        <v>1</v>
+      </c>
+      <c r="L6" s="75">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12">
+      <c r="A7" s="81"/>
+      <c r="B7" s="81" t="s">
+        <v>84</v>
+      </c>
+      <c r="C7" s="76">
+        <v>0.5</v>
+      </c>
+      <c r="D7" s="76">
+        <v>0</v>
+      </c>
+      <c r="E7" s="76">
+        <v>0.98810458970000004</v>
+      </c>
+      <c r="F7" s="76">
+        <v>0</v>
+      </c>
+      <c r="G7" s="76">
+        <v>0</v>
+      </c>
+      <c r="H7" s="76">
+        <v>0</v>
+      </c>
+      <c r="I7" s="76">
+        <v>0</v>
+      </c>
+      <c r="J7" s="76">
+        <v>0</v>
+      </c>
+      <c r="K7" s="76">
+        <v>1</v>
+      </c>
+      <c r="L7" s="77">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12">
+      <c r="A8" s="79" t="s">
+        <v>30</v>
+      </c>
+      <c r="B8" s="79" t="s">
+        <v>80</v>
+      </c>
+      <c r="C8" s="72">
+        <v>0.51045209260000002</v>
+      </c>
+      <c r="D8" s="72">
+        <v>1.420647802E-2</v>
+      </c>
+      <c r="E8" s="72">
+        <v>0.95652194580000005</v>
+      </c>
+      <c r="F8" s="72">
+        <v>1.553847671E-2</v>
+      </c>
+      <c r="G8" s="72">
+        <v>2.4088161779999999E-2</v>
+      </c>
+      <c r="H8" s="72">
+        <v>2.1048966119999998E-2</v>
+      </c>
+      <c r="I8" s="72">
+        <v>3.9525691699999997E-2</v>
+      </c>
+      <c r="J8" s="72">
+        <v>4.340083736E-2</v>
+      </c>
+      <c r="K8" s="72">
+        <v>0.98137849349999995</v>
+      </c>
+      <c r="L8" s="73">
+        <v>1.7072566769999999E-2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12">
+      <c r="A9" s="80"/>
+      <c r="B9" s="82" t="s">
+        <v>85</v>
+      </c>
+      <c r="C9" s="74">
+        <v>0.5</v>
+      </c>
+      <c r="D9" s="74">
+        <v>0</v>
+      </c>
+      <c r="E9" s="74">
+        <v>0.97359220170000005</v>
+      </c>
+      <c r="F9" s="74">
+        <v>0</v>
+      </c>
+      <c r="G9" s="74">
+        <v>0</v>
+      </c>
+      <c r="H9" s="74">
+        <v>0</v>
+      </c>
+      <c r="I9" s="74">
+        <v>0</v>
+      </c>
+      <c r="J9" s="74">
+        <v>0</v>
+      </c>
+      <c r="K9" s="74">
+        <v>1</v>
+      </c>
+      <c r="L9" s="75">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12">
+      <c r="A10" s="80"/>
+      <c r="B10" s="80" t="s">
+        <v>83</v>
+      </c>
+      <c r="C10" s="74">
+        <v>0.5</v>
+      </c>
+      <c r="D10" s="74">
+        <v>0</v>
+      </c>
+      <c r="E10" s="74">
+        <v>0.97359220170000005</v>
+      </c>
+      <c r="F10" s="74">
+        <v>0</v>
+      </c>
+      <c r="G10" s="74">
+        <v>0</v>
+      </c>
+      <c r="H10" s="74">
+        <v>0</v>
+      </c>
+      <c r="I10" s="74">
+        <v>0</v>
+      </c>
+      <c r="J10" s="74">
+        <v>0</v>
+      </c>
+      <c r="K10" s="74">
+        <v>1</v>
+      </c>
+      <c r="L10" s="75">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12">
+      <c r="A11" s="80"/>
+      <c r="B11" s="80" t="s">
+        <v>82</v>
+      </c>
+      <c r="C11" s="74">
+        <v>0.4997889023</v>
+      </c>
+      <c r="D11" s="74">
+        <v>4.9348362320000003E-4</v>
+      </c>
+      <c r="E11" s="74">
+        <v>0.97318092089999997</v>
+      </c>
+      <c r="F11" s="74">
+        <v>9.6145222939999998E-4</v>
+      </c>
+      <c r="G11" s="74">
+        <v>0</v>
+      </c>
+      <c r="H11" s="74">
+        <v>0</v>
+      </c>
+      <c r="I11" s="74">
+        <v>0</v>
+      </c>
+      <c r="J11" s="74">
+        <v>0</v>
+      </c>
+      <c r="K11" s="74">
+        <v>0.99957780460000001</v>
+      </c>
+      <c r="L11" s="75">
+        <v>9.8696724640000007E-4</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12">
+      <c r="A12" s="80"/>
+      <c r="B12" s="80" t="s">
+        <v>81</v>
+      </c>
+      <c r="C12" s="74">
+        <v>0.5</v>
+      </c>
+      <c r="D12" s="74">
+        <v>0</v>
+      </c>
+      <c r="E12" s="74">
+        <v>0.97359220170000005</v>
+      </c>
+      <c r="F12" s="74">
+        <v>0</v>
+      </c>
+      <c r="G12" s="74">
+        <v>0</v>
+      </c>
+      <c r="H12" s="74">
+        <v>0</v>
+      </c>
+      <c r="I12" s="74">
+        <v>0</v>
+      </c>
+      <c r="J12" s="74">
+        <v>0</v>
+      </c>
+      <c r="K12" s="74">
+        <v>1</v>
+      </c>
+      <c r="L12" s="75">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12">
+      <c r="A13" s="81"/>
+      <c r="B13" s="81" t="s">
+        <v>84</v>
+      </c>
+      <c r="C13" s="76">
+        <v>0.5</v>
+      </c>
+      <c r="D13" s="76">
+        <v>0</v>
+      </c>
+      <c r="E13" s="76">
+        <v>0.97359220170000005</v>
+      </c>
+      <c r="F13" s="76">
+        <v>0</v>
+      </c>
+      <c r="G13" s="76">
+        <v>0</v>
+      </c>
+      <c r="H13" s="76">
+        <v>0</v>
+      </c>
+      <c r="I13" s="76">
+        <v>0</v>
+      </c>
+      <c r="J13" s="76">
+        <v>0</v>
+      </c>
+      <c r="K13" s="76">
+        <v>1</v>
+      </c>
+      <c r="L13" s="77">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12">
+      <c r="A14" s="79" t="s">
+        <v>32</v>
+      </c>
+      <c r="B14" s="82" t="s">
+        <v>85</v>
+      </c>
+      <c r="C14" s="72">
+        <v>0.65806684019999995</v>
+      </c>
+      <c r="D14" s="72">
+        <v>7.2973800120000001E-2</v>
+      </c>
+      <c r="E14" s="72">
+        <v>0.90364181659999998</v>
+      </c>
+      <c r="F14" s="72">
+        <v>4.5378007120000001E-2</v>
+      </c>
+      <c r="G14" s="72">
+        <v>3.0278070010000002E-2</v>
+      </c>
+      <c r="H14" s="72">
+        <v>1.5961233049999999E-2</v>
+      </c>
+      <c r="I14" s="72">
+        <v>0.4080645161</v>
+      </c>
+      <c r="J14" s="72">
+        <v>0.1854721829</v>
+      </c>
+      <c r="K14" s="72">
+        <v>0.90806916429999995</v>
+      </c>
+      <c r="L14" s="73">
+        <v>4.722630874E-2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12">
+      <c r="A15" s="80"/>
+      <c r="B15" s="80" t="s">
+        <v>80</v>
+      </c>
+      <c r="C15" s="74">
+        <v>0.56444222369999997</v>
+      </c>
+      <c r="D15" s="74">
+        <v>5.0401044890000003E-2</v>
+      </c>
+      <c r="E15" s="74">
+        <v>0.93668951730000005</v>
+      </c>
+      <c r="F15" s="74">
+        <v>5.4301813079999997E-2</v>
+      </c>
+      <c r="G15" s="74">
+        <v>1.7110157460000001E-2</v>
+      </c>
+      <c r="H15" s="74">
+        <v>1.1428109049999999E-2</v>
+      </c>
+      <c r="I15" s="74">
+        <v>0.18548387099999999</v>
+      </c>
+      <c r="J15" s="74">
+        <v>0.15475094589999999</v>
+      </c>
+      <c r="K15" s="74">
+        <v>0.94340057639999997</v>
+      </c>
+      <c r="L15" s="75">
+        <v>5.6133893480000002E-2</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12">
+      <c r="A16" s="80"/>
+      <c r="B16" s="80" t="s">
+        <v>82</v>
+      </c>
+      <c r="C16" s="74">
+        <v>0.5</v>
+      </c>
+      <c r="D16" s="74">
+        <v>0</v>
+      </c>
+      <c r="E16" s="74">
+        <v>0.99114538699999999</v>
+      </c>
+      <c r="F16" s="74">
+        <v>0</v>
+      </c>
+      <c r="G16" s="74">
+        <v>0</v>
+      </c>
+      <c r="H16" s="74">
+        <v>0</v>
+      </c>
+      <c r="I16" s="74">
+        <v>0</v>
+      </c>
+      <c r="J16" s="74">
+        <v>0</v>
+      </c>
+      <c r="K16" s="74">
+        <v>1</v>
+      </c>
+      <c r="L16" s="75">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12">
+      <c r="A17" s="80"/>
+      <c r="B17" s="80" t="s">
+        <v>81</v>
+      </c>
+      <c r="C17" s="74">
+        <v>0.5</v>
+      </c>
+      <c r="D17" s="74">
+        <v>0</v>
+      </c>
+      <c r="E17" s="74">
+        <v>0.84647817459999997</v>
+      </c>
+      <c r="F17" s="74">
+        <v>0</v>
+      </c>
+      <c r="G17" s="74">
+        <v>0</v>
+      </c>
+      <c r="H17" s="74">
+        <v>0</v>
+      </c>
+      <c r="I17" s="74">
+        <v>0</v>
+      </c>
+      <c r="J17" s="74">
+        <v>0</v>
+      </c>
+      <c r="K17" s="74">
+        <v>1</v>
+      </c>
+      <c r="L17" s="75">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12">
+      <c r="A18" s="80"/>
+      <c r="B18" s="80" t="s">
+        <v>83</v>
+      </c>
+      <c r="C18" s="74">
+        <v>0.5</v>
+      </c>
+      <c r="D18" s="74">
+        <v>0</v>
+      </c>
+      <c r="E18" s="74">
+        <v>0.99114538699999999</v>
+      </c>
+      <c r="F18" s="74">
+        <v>0</v>
+      </c>
+      <c r="G18" s="74">
+        <v>0</v>
+      </c>
+      <c r="H18" s="74">
+        <v>0</v>
+      </c>
+      <c r="I18" s="74">
+        <v>0</v>
+      </c>
+      <c r="J18" s="74">
+        <v>0</v>
+      </c>
+      <c r="K18" s="74">
+        <v>1</v>
+      </c>
+      <c r="L18" s="75">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12">
+      <c r="A19" s="81"/>
+      <c r="B19" s="81" t="s">
+        <v>84</v>
+      </c>
+      <c r="C19" s="76">
+        <v>0.5</v>
+      </c>
+      <c r="D19" s="76">
+        <v>0</v>
+      </c>
+      <c r="E19" s="76">
+        <v>0.99114538699999999</v>
+      </c>
+      <c r="F19" s="76">
+        <v>0</v>
+      </c>
+      <c r="G19" s="76">
+        <v>0</v>
+      </c>
+      <c r="H19" s="76">
+        <v>0</v>
+      </c>
+      <c r="I19" s="76">
+        <v>0</v>
+      </c>
+      <c r="J19" s="76">
+        <v>0</v>
+      </c>
+      <c r="K19" s="76">
+        <v>1</v>
+      </c>
+      <c r="L19" s="77">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12">
+      <c r="A20" s="79" t="s">
+        <v>21</v>
+      </c>
+      <c r="B20" s="79" t="s">
+        <v>82</v>
+      </c>
+      <c r="C20" s="72">
+        <v>0.56156623790000004</v>
+      </c>
+      <c r="D20" s="72">
+        <v>7.9767480970000006E-3</v>
+      </c>
+      <c r="E20" s="72">
+        <v>0.48873903400000002</v>
+      </c>
+      <c r="F20" s="72">
+        <v>3.1899364040000003E-2</v>
+      </c>
+      <c r="G20" s="72">
+        <v>0.24876614720000001</v>
+      </c>
+      <c r="H20" s="72">
+        <v>6.60681681E-3</v>
+      </c>
+      <c r="I20" s="72">
+        <v>0.6884106686</v>
+      </c>
+      <c r="J20" s="72">
+        <v>4.397029408E-2</v>
+      </c>
+      <c r="K20" s="72">
+        <v>0.43472180710000002</v>
+      </c>
+      <c r="L20" s="73">
+        <v>5.1772101680000002E-2</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12">
+      <c r="A21" s="80"/>
+      <c r="B21" s="80" t="s">
+        <v>80</v>
+      </c>
+      <c r="C21" s="74">
+        <v>0.50339840889999998</v>
+      </c>
+      <c r="D21" s="74">
+        <v>6.557784243E-3</v>
+      </c>
+      <c r="E21" s="74">
+        <v>0.78450942229999998</v>
+      </c>
+      <c r="F21" s="74">
+        <v>6.6074839290000001E-3</v>
+      </c>
+      <c r="G21" s="74">
+        <v>0.52690774259999995</v>
+      </c>
+      <c r="H21" s="74">
+        <v>0.19228775319999999</v>
+      </c>
+      <c r="I21" s="74">
+        <v>1.378398477E-2</v>
+      </c>
+      <c r="J21" s="74">
+        <v>2.942301625E-2</v>
+      </c>
+      <c r="K21" s="74">
+        <v>0.99301283299999998</v>
+      </c>
+      <c r="L21" s="75">
+        <v>1.6341350019999999E-2</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12">
+      <c r="A22" s="80"/>
+      <c r="B22" s="82" t="s">
+        <v>85</v>
+      </c>
+      <c r="C22" s="74">
+        <v>0.50094485639999997</v>
+      </c>
+      <c r="D22" s="74">
+        <v>3.0184013689999998E-3</v>
+      </c>
+      <c r="E22" s="74">
+        <v>0.78372297909999999</v>
+      </c>
+      <c r="F22" s="74">
+        <v>7.52478587E-3</v>
+      </c>
+      <c r="G22" s="74">
+        <v>0.1268482457</v>
+      </c>
+      <c r="H22" s="74">
+        <v>0.2317008793</v>
+      </c>
+      <c r="I22" s="74">
+        <v>8.4263450479999998E-3</v>
+      </c>
+      <c r="J22" s="74">
+        <v>1.7637927420000001E-2</v>
+      </c>
+      <c r="K22" s="74">
+        <v>0.99346336769999999</v>
+      </c>
+      <c r="L22" s="75">
+        <v>1.3997602119999999E-2</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12">
+      <c r="A23" s="80"/>
+      <c r="B23" s="80" t="s">
+        <v>81</v>
+      </c>
+      <c r="C23" s="74">
+        <v>0.5</v>
+      </c>
+      <c r="D23" s="74">
+        <v>0</v>
+      </c>
+      <c r="E23" s="74">
+        <v>0.99114538699999999</v>
+      </c>
+      <c r="F23" s="74">
+        <v>0</v>
+      </c>
+      <c r="G23" s="74">
+        <v>0</v>
+      </c>
+      <c r="H23" s="74">
+        <v>0</v>
+      </c>
+      <c r="I23" s="74">
+        <v>0</v>
+      </c>
+      <c r="J23" s="74">
+        <v>0</v>
+      </c>
+      <c r="K23" s="74">
+        <v>1</v>
+      </c>
+      <c r="L23" s="75">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12">
+      <c r="A24" s="80"/>
+      <c r="B24" s="80" t="s">
+        <v>83</v>
+      </c>
+      <c r="C24" s="74">
+        <v>0.50094485639999997</v>
+      </c>
+      <c r="D24" s="74">
+        <v>3.0184013689999998E-3</v>
+      </c>
+      <c r="E24" s="74">
+        <v>0.78372297909999999</v>
+      </c>
+      <c r="F24" s="74">
+        <v>7.52478587E-3</v>
+      </c>
+      <c r="G24" s="74">
+        <v>0.1268482457</v>
+      </c>
+      <c r="H24" s="74">
+        <v>0.2317008793</v>
+      </c>
+      <c r="I24" s="74">
+        <v>8.4263450479999998E-3</v>
+      </c>
+      <c r="J24" s="74">
+        <v>1.7637927420000001E-2</v>
+      </c>
+      <c r="K24" s="74">
+        <v>0.99346336769999999</v>
+      </c>
+      <c r="L24" s="75">
+        <v>1.3997602119999999E-2</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12">
+      <c r="A25" s="81"/>
+      <c r="B25" s="81" t="s">
+        <v>84</v>
+      </c>
+      <c r="C25" s="76">
+        <v>0.50312129179999998</v>
+      </c>
+      <c r="D25" s="76">
+        <v>4.5376267750000003E-3</v>
+      </c>
+      <c r="E25" s="76">
+        <v>0.78550123940000005</v>
+      </c>
+      <c r="F25" s="76">
+        <v>2.0141718729999999E-3</v>
+      </c>
+      <c r="G25" s="76">
+        <v>0.51509397400000001</v>
+      </c>
+      <c r="H25" s="76">
+        <v>0.13185474450000001</v>
+      </c>
+      <c r="I25" s="76">
+        <v>1.129679988E-2</v>
+      </c>
+      <c r="J25" s="76">
+        <v>1.5919054410000001E-2</v>
+      </c>
+      <c r="K25" s="76">
+        <v>0.99494578379999998</v>
+      </c>
+      <c r="L25" s="77">
+        <v>6.8552873149999999E-3</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12">
+      <c r="A26" s="79" t="s">
+        <v>20</v>
+      </c>
+      <c r="B26" s="79" t="s">
+        <v>80</v>
+      </c>
+      <c r="C26" s="72">
+        <v>0.50102703540000004</v>
+      </c>
+      <c r="D26" s="72">
+        <v>1.7853868889999999E-2</v>
+      </c>
+      <c r="E26" s="72">
+        <v>0.83602017200000001</v>
+      </c>
+      <c r="F26" s="72">
+        <v>9.057108203E-3</v>
+      </c>
+      <c r="G26" s="72">
+        <v>8.3333333329999995E-2</v>
+      </c>
+      <c r="H26" s="72">
+        <v>0.1443375673</v>
+      </c>
+      <c r="I26" s="72">
+        <v>1.754385965E-2</v>
+      </c>
+      <c r="J26" s="72">
+        <v>3.0386856269999998E-2</v>
+      </c>
+      <c r="K26" s="72">
+        <v>0.98451021110000003</v>
+      </c>
+      <c r="L26" s="73">
+        <v>5.321031201E-3</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12">
+      <c r="A27" s="80"/>
+      <c r="B27" s="82" t="s">
+        <v>85</v>
+      </c>
+      <c r="C27" s="74">
+        <v>0.5</v>
+      </c>
+      <c r="D27" s="74">
+        <v>0</v>
+      </c>
+      <c r="E27" s="74">
+        <v>0.84647817459999997</v>
+      </c>
+      <c r="F27" s="74">
+        <v>0</v>
+      </c>
+      <c r="G27" s="74">
+        <v>0</v>
+      </c>
+      <c r="H27" s="74">
+        <v>0</v>
+      </c>
+      <c r="I27" s="74">
+        <v>0</v>
+      </c>
+      <c r="J27" s="74">
+        <v>0</v>
+      </c>
+      <c r="K27" s="74">
+        <v>1</v>
+      </c>
+      <c r="L27" s="75">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12">
+      <c r="A28" s="80"/>
+      <c r="B28" s="80" t="s">
+        <v>83</v>
+      </c>
+      <c r="C28" s="74">
+        <v>0.5</v>
+      </c>
+      <c r="D28" s="74">
+        <v>0</v>
+      </c>
+      <c r="E28" s="74">
+        <v>0.84647817459999997</v>
+      </c>
+      <c r="F28" s="74">
+        <v>0</v>
+      </c>
+      <c r="G28" s="74">
+        <v>0</v>
+      </c>
+      <c r="H28" s="74">
+        <v>0</v>
+      </c>
+      <c r="I28" s="74">
+        <v>0</v>
+      </c>
+      <c r="J28" s="74">
+        <v>0</v>
+      </c>
+      <c r="K28" s="74">
+        <v>1</v>
+      </c>
+      <c r="L28" s="75">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12">
+      <c r="A29" s="80"/>
+      <c r="B29" s="80" t="s">
+        <v>81</v>
+      </c>
+      <c r="C29" s="74">
+        <v>0.5</v>
+      </c>
+      <c r="D29" s="74">
+        <v>0</v>
+      </c>
+      <c r="E29" s="74">
+        <v>0.787073625</v>
+      </c>
+      <c r="F29" s="74">
+        <v>0</v>
+      </c>
+      <c r="G29" s="74">
+        <v>0</v>
+      </c>
+      <c r="H29" s="74">
+        <v>0</v>
+      </c>
+      <c r="I29" s="74">
+        <v>0</v>
+      </c>
+      <c r="J29" s="74">
+        <v>0</v>
+      </c>
+      <c r="K29" s="74">
+        <v>1</v>
+      </c>
+      <c r="L29" s="75">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:12">
+      <c r="A30" s="80"/>
+      <c r="B30" s="80" t="s">
+        <v>84</v>
+      </c>
+      <c r="C30" s="74">
+        <v>0.5</v>
+      </c>
+      <c r="D30" s="74">
+        <v>0</v>
+      </c>
+      <c r="E30" s="74">
+        <v>0.84647817459999997</v>
+      </c>
+      <c r="F30" s="74">
+        <v>0</v>
+      </c>
+      <c r="G30" s="74">
+        <v>0</v>
+      </c>
+      <c r="H30" s="74">
+        <v>0</v>
+      </c>
+      <c r="I30" s="74">
+        <v>0</v>
+      </c>
+      <c r="J30" s="74">
+        <v>0</v>
+      </c>
+      <c r="K30" s="74">
+        <v>1</v>
+      </c>
+      <c r="L30" s="75">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:12">
+      <c r="A31" s="81"/>
+      <c r="B31" s="81" t="s">
+        <v>82</v>
+      </c>
+      <c r="C31" s="76">
+        <v>0.49663385920000003</v>
+      </c>
+      <c r="D31" s="76">
+        <v>1.284004519E-2</v>
+      </c>
+      <c r="E31" s="76">
+        <v>0.80603091930000004</v>
+      </c>
+      <c r="F31" s="76">
+        <v>3.0332321839999999E-2</v>
+      </c>
+      <c r="G31" s="76">
+        <v>0.11011904760000001</v>
+      </c>
+      <c r="H31" s="76">
+        <v>4.2194782379999997E-2</v>
+      </c>
+      <c r="I31" s="76">
+        <v>5.0438596490000001E-2</v>
+      </c>
+      <c r="J31" s="76">
+        <v>2.434506857E-2</v>
+      </c>
+      <c r="K31" s="76">
+        <v>0.94282912200000002</v>
+      </c>
+      <c r="L31" s="77">
+        <v>3.9357609740000001E-2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>